<commit_message>
feat: added updated BOM, new controller code for better button debouncing and a version of the controller code that supports calibration for the joysticks.
</commit_message>
<xml_diff>
--- a/Version WIP/Aegis 2 BOM.xlsx
+++ b/Version WIP/Aegis 2 BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djuckett\Dropbox\Projects\Aegis 2\Aegis-2\Version WIP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jucke\Dropbox\Projects\Aegis 2\Aegis-2\Version WIP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E7D823-75A2-479A-810E-653DB9E74DF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29D3D4B-318A-4E78-ABDD-27C0D878FA11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{93BD1906-D6D6-45EE-A20C-B1437B097662}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{93BD1906-D6D6-45EE-A20C-B1437B097662}"/>
   </bookViews>
   <sheets>
     <sheet name="Main Board" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="320">
   <si>
     <t>Qty</t>
   </si>
@@ -141,9 +141,6 @@
     <t>https://www.digikey.com/en/products/detail/c-k/KSS331GLFS/417674?s=N4IgTCBcDaINIGUEGZkEYDiAZAYgkAugL5A</t>
   </si>
   <si>
-    <t>https://www.aliexpress.com/item/33049485687.html?spm=a2g0s.9042311.0.0.1b124c4d3HPSEF</t>
-  </si>
-  <si>
     <t>Mezzanine Connector (RP4)</t>
   </si>
   <si>
@@ -324,9 +321,6 @@
     <t>Res 15K (603)</t>
   </si>
   <si>
-    <t>Cap 100uF (603)</t>
-  </si>
-  <si>
     <t>Inductors</t>
   </si>
   <si>
@@ -384,9 +378,6 @@
     <t>Cap 0.1uf (805 Film)</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/cornell-dubilier-electronics-cde/FCA0805C104M-J2/1924083</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/vishay-sprague/T55B227M6R3C0035/5357197</t>
   </si>
   <si>
@@ -525,9 +516,6 @@
     <t>https://www.digikey.com/en/products/detail/maxim-integrated/MAX98306ETD-T/2708795</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/avx-corporation/F980J107MMAAXE/5957626?s=N4IgjCBcpgbFoDGUBmBDANgZwKYBoQB7KAbRAGYBOAJgBZ4BdAgBwBcoQBlVgJwEsAdgHMQAXwJhKADkoIQySOmz4ipEAAYQTEGw7d%2BwsQWrras6DvaQQAVQF9WAeRQBZHGiwBXHjhAFPHACtAGJ%2BIAC2ghxg6poE4WgAHtGxRiAmAOzmSKiYuATEkGSwAGphsAB05GUEUjXg6vVgAKxNpWEm9dStYeSNvT0EtP0EzSMgsONg3WXautZ2Ds5uHt6%2BouLpaohozGiIDoQ8WqJAA</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/cnc-tech/2001-1-2-21-00-BK/4867021?s=N4IgTCBcDa4AxwIwFoVmWFDkCEDSIAugL5A</t>
   </si>
   <si>
@@ -765,9 +753,6 @@
     <t>JOYSTICK_L</t>
   </si>
   <si>
-    <t>https://www.sparkfun.com/products/13305</t>
-  </si>
-  <si>
     <t>CNTRL_BRD_CONN</t>
   </si>
   <si>
@@ -783,9 +768,6 @@
     <t>HEAD_AMP</t>
   </si>
   <si>
-    <t>Audio DAC</t>
-  </si>
-  <si>
     <t>Speaker Amplifier</t>
   </si>
   <si>
@@ -843,9 +825,6 @@
     <t>BUT_START</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/mitsumi-electric-company-ltd/R-667834/11591283</t>
-  </si>
-  <si>
     <t>Tactile Switches</t>
   </si>
   <si>
@@ -864,9 +843,6 @@
     <t>SHLD_BUT_L</t>
   </si>
   <si>
-    <t>https://www.ebay.com/itm/354618455099?chn=ps&amp;var=623990696410&amp;_trkparms=ispr%3D1&amp;amdata=enc%3A1Zk6c1fiYQTmjnu1i-GLg_w51&amp;norover=1&amp;mkevt=1&amp;mkrid=711-117182-37290-0&amp;mkcid=2&amp;mkscid=101&amp;itemid=623990696410_354618455099&amp;targetid=1584739238534&amp;device=c&amp;mktype=&amp;googleloc=9016965&amp;poi=&amp;campaignid=15275224983&amp;mkgroupid=131097072938&amp;rlsatarget=pla-1584739238534&amp;abcId=9300697&amp;merchantid=633191918&amp;gclid=CjwKCAjw3ueiBhBmEiwA4BhspPro6b1IzauVdwTaQfRWhvR-m2RbObJTIP_17MVH22aw1EJwAAuf9hoCW1kQAvD_BwE</t>
-  </si>
-  <si>
     <t>R1, R2, R3, R4, R5, R6, R7, R8</t>
   </si>
   <si>
@@ -927,15 +903,9 @@
     <t>JOYSTICK_R</t>
   </si>
   <si>
-    <t>7" Screen</t>
-  </si>
-  <si>
     <t>SCREEN</t>
   </si>
   <si>
-    <t>https://www.aliexpress.us/item/2251832639945508.html?spm=a2g0o.order_list.order_list_main.31.1e141802tcsJdw&amp;gatewayAdapt=glo2usa</t>
-  </si>
-  <si>
     <t>SCREEN_CABLE</t>
   </si>
   <si>
@@ -972,19 +942,61 @@
     <t>BUTTONS</t>
   </si>
   <si>
-    <t>https://www.aliexpress.us/item/3256802895965671.html?spm=a2g0o.order_list.order_list_main.111.675d1802dWILfE&amp;gatewayAdapt=glo2usa4itemAdapt</t>
-  </si>
-  <si>
     <t>Cap  330 nF (603)</t>
   </si>
   <si>
-    <t>https://www.aliexpress.us/item/3256803228333750.html?spm=a2g0o.productlist.main.1.27357aedfOveIi&amp;algo_pvid=b9289e00-9e59-4056-b51a-43910fcea86f&amp;algo_exp_id=b9289e00-9e59-4056-b51a-43910fcea86f-0&amp;pdp_npi=3%40dis%21USD%2111.59%219.62%21%21%21%21%21%40212278bd16865808440348119d07cd%2112000025683190881%21sea%21US%211888726260&amp;curPageLogUid=DbxWuEx0YQy9</t>
-  </si>
-  <si>
     <t>R4</t>
   </si>
   <si>
     <t>R3, R6, R7, R8, R9, R10, R11, R12, R13, R14, R15</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.us/item/3256809705127240.html?spm=a2g0o.productlist.main.1.33ae7aedIgg3oA&amp;algo_pvid=88988f2f-f7e9-46bb-837c-9555500715a3&amp;algo_exp_id=88988f2f-f7e9-46bb-837c-9555500715a3-0&amp;pdp_ext_f=%7B%22order%22%3A%22-1%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21USD%2116.66%2113.50%21%21%21116.81%2194.62%21%402101d6fe17655858242445266eb68f%2112000050496962191%21sea%21US%211888726260%21X%211%210%21n_tag%3A-29919%3Bd%3A838ad40a%3Bm03_new_user%3A-29895&amp;curPageLogUid=XkGiW34YB1yB&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005009891441992%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.us/item/3256807988088764.html?spm=a2g0o.productlist.main.1.7a0f5bc1S5Su9A&amp;algo_pvid=794f334d-d3fa-47ba-95b1-6e953b720bd3&amp;algo_exp_id=794f334d-d3fa-47ba-95b1-6e953b720bd3-0&amp;pdp_ext_f=%7B%22order%22%3A%221%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21USD%2143.51%2140.03%21%21%21305.10%21280.69%21%40210328c017655859840498892ec076%2112000044109156759%21sea%21US%211888726260%21X%211%210%21n_tag%3A-29919%3Bd%3A838ad40a%3Bm03_new_user%3A-29895&amp;curPageLogUid=1FE7APp9S0mD&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005008174403516%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>7" Screen (LT070ME05000)</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.us/item/3256802569830553.html?spm=a2g0o.productlist.main.2.5faf34c2cTAIDx&amp;algo_pvid=829a0b61-830f-4297-94c2-714e6da0c128&amp;algo_exp_id=829a0b61-830f-4297-94c2-714e6da0c128-1&amp;pdp_ext_f=%7B%22order%22%3A%229%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21USD%2114.81%2110.81%21%21%2114.81%2110.81%21%40210328db17655863106172233e5944%2112000021992697124%21sea%21US%211888726260%21X%211%210%21n_tag%3A-29919%3Bd%3A838ad40a%3Bm03_new_user%3A-29895&amp;curPageLogUid=qyGqs3tZlrvy&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005002756145305%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>https://www.radwell.com/Buy/PJRC/PJRC/TEENSY-LC?source=GoogleShopping&amp;IgnoreRedirect=true&amp;ItemSingleId=247864851&amp;viewAll=true&amp;gad_source=1&amp;gad_campaignid=22852792497&amp;gbraid=0AAAAADHiFo9Uj7T_r5m5FHOHMbx5oB4zP&amp;gclid=CjwKCAiAl-_JBhBjEiwAn3rN7SL6vEIvBjDUtx_Nw4cJozM8A1PH4EA-2v5AfZuOu86_ZsEooGIanRoCcPYQAvD_BwE</t>
+  </si>
+  <si>
+    <t>Teensy 4 as a drop in replacement for Teensy LC</t>
+  </si>
+  <si>
+    <t>https://www.adafruit.com/product/4323?gad_source=1&amp;gad_campaignid=21079227318&amp;gbraid=0AAAAADx9JvTOdF_aT3h3708M5CBet26Hr&amp;gclid=CjwKCAiAl-_JBhBjEiwAn3rN7XLPsGYGNH3YIMym7HS72tDJYnModsQCM9-hXBlViEzHjtH69iA4jBoCGs0QAvD_BwE</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/mitsumi-electric-company-ltd/R-667837/11591258</t>
+  </si>
+  <si>
+    <t>https://www.ebay.com/itm/376766825242?_trkparms=amclksrc%3DITM%26aid%3D1110006%26algo%3DHOMESPLICE.SIM%26ao%3D1%26asc%3D20200818143230%26meid%3D8d5e1d7907b14e738db13161ceb94768%26pid%3D101224%26rk%3D2%26rkt%3D5%26sd%3D354618455099%26itm%3D376766825242%26pmt%3D1%26noa%3D1%26pg%3D2332490%26algv%3DDefaultOrganicWebV9BertRefreshRankerWithCassiniEmbRecall%26brand%3DUnbranded&amp;_trksid=p2332490.c101224.m-1</t>
+  </si>
+  <si>
+    <t>Audio DAC (UDA1334ATS)</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.us/item/3256810009871385.html?spm=a2g0o.productlist.main.4.232b57aag1HAwF&amp;aem_p4p_detail=2025121217024213882094407348440000453386&amp;algo_pvid=da82ab22-cc01-43c5-8046-5395ceff02c6&amp;algo_exp_id=da82ab22-cc01-43c5-8046-5395ceff02c6-3&amp;pdp_ext_f=%7B%22order%22%3A%221%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21USD%218.22%216.41%21%21%218.22%216.41%21%40210311c217655877628664897ea4af%2112000051487159061%21sea%21US%211888726260%21X%211%210%21n_tag%3A-29919%3Bd%3A838ad40a%3Bm03_new_user%3A-29895&amp;curPageLogUid=7ITlGC4Lj2uC&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005010196186137%7C_p_origin_prod%3A&amp;search_p4p_id=2025121217024213882094407348440000453386_1</t>
+  </si>
+  <si>
+    <t>https://www.ebay.com/itm/376766825242?_trkparms=amclksrc%3DITM%26aid%3D1110006%26algo%3DHOMESPLICE.SIM%26ao%3D1%26asc%3D20200818143230%26meid%3D96ffe1439d9846bd91e6bfcdf3f3581d%26pid%3D101224%26rk%3D2%26rkt%3D5%26sd%3D354618455099%26itm%3D376766825242%26pmt%3D1%26noa%3D1%26pg%3D2332490%26algv%3DDefaultOrganicWebV9BertRefreshRankerWithCassiniEmbRecall%26brand%3DUnbranded&amp;_trksid=p2332490.c101224.m-1</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/murata-electronics/GRT188R61A106KE13D/5417012</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/rubycon/25MU104KZ22012/9951730</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/vishay-sprague/298D107X06R3P2T/1973815</t>
+  </si>
+  <si>
+    <t>Cap 100uF (805)</t>
   </si>
 </sst>
 </file>
@@ -1067,7 +1079,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1099,6 +1111,8 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1118,9 +1132,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1158,7 +1172,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1264,7 +1278,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1406,7 +1420,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1428,7 +1442,7 @@
         <v>21</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -1445,7 +1459,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" s="8"/>
     </row>
@@ -1454,7 +1468,7 @@
         <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -1475,7 +1489,7 @@
         <v>20</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1493,10 +1507,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1509,15 +1523,15 @@
         <v>2.4300000000000002</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1530,15 +1544,15 @@
         <v>3.37</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -1551,15 +1565,15 @@
         <v>0.5</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1572,15 +1586,15 @@
         <v>0.2</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -1593,15 +1607,15 @@
         <v>1.86</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1614,15 +1628,15 @@
         <v>0.7</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1635,7 +1649,7 @@
         <v>6.04</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1643,7 +1657,7 @@
     </row>
     <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B13" s="8"/>
     </row>
@@ -1652,7 +1666,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1670,7 +1684,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" s="8"/>
     </row>
@@ -1679,7 +1693,7 @@
         <v>8</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C17">
         <v>2</v>
@@ -1692,15 +1706,15 @@
         <v>3.8</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1713,15 +1727,15 @@
         <v>3.87</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1734,15 +1748,15 @@
         <v>0.46</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1755,15 +1769,15 @@
         <v>0.59</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1776,12 +1790,12 @@
         <v>0.8</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B23" s="8"/>
     </row>
@@ -1790,7 +1804,7 @@
         <v>9</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1803,15 +1817,15 @@
         <v>1.94</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -1824,21 +1838,21 @@
         <v>0.4</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B27" s="8"/>
     </row>
     <row r="28" spans="1:6" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1851,15 +1865,15 @@
         <v>3</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -1872,7 +1886,7 @@
         <v>0.92</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -1880,15 +1894,15 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1901,7 +1915,7 @@
         <v>1.38</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -1909,16 +1923,16 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B34" s="8"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -1936,10 +1950,10 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -1952,7 +1966,7 @@
         <v>4.03</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -1960,16 +1974,16 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B38" s="8"/>
     </row>
     <row r="39" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C39">
         <v>2</v>
@@ -1987,10 +2001,10 @@
     </row>
     <row r="40" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C40">
         <v>1</v>
@@ -2003,7 +2017,7 @@
         <v>2.12</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -2012,16 +2026,16 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B42" s="8"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -2034,7 +2048,7 @@
         <v>0.43</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -2042,7 +2056,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B45" s="8"/>
       <c r="F45" s="5"/>
@@ -2052,7 +2066,7 @@
         <v>16</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -2074,17 +2088,17 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B48" s="1"/>
       <c r="F48" s="5"/>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -2097,15 +2111,15 @@
         <v>0.94</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -2118,15 +2132,15 @@
         <v>0.11</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -2139,15 +2153,15 @@
         <v>0.18</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -2165,10 +2179,10 @@
     </row>
     <row r="53" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="C53">
         <v>11</v>
@@ -2186,10 +2200,10 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C54">
         <v>2</v>
@@ -2202,15 +2216,15 @@
         <v>0.22</v>
       </c>
       <c r="F54" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C55">
         <v>1</v>
@@ -2223,15 +2237,15 @@
         <v>0.1</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C56">
         <v>4</v>
@@ -2244,15 +2258,15 @@
         <v>0.4</v>
       </c>
       <c r="F56" s="5" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -2265,15 +2279,15 @@
         <v>0.1</v>
       </c>
       <c r="F57" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="11" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -2286,15 +2300,15 @@
         <v>0.1</v>
       </c>
       <c r="F58" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -2307,7 +2321,7 @@
         <v>0.1</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -2317,17 +2331,17 @@
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B61" s="1"/>
       <c r="F61" s="5"/>
     </row>
     <row r="62" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="11" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C62">
         <v>2</v>
@@ -2340,15 +2354,15 @@
         <v>0.2</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="63" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="11" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -2361,15 +2375,15 @@
         <v>0.1</v>
       </c>
       <c r="F63" s="5" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="64" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="11" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="C64">
         <v>1</v>
@@ -2382,15 +2396,15 @@
         <v>0.1</v>
       </c>
       <c r="F64" s="5" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C65">
         <v>1</v>
@@ -2408,10 +2422,10 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C66">
         <v>7</v>
@@ -2424,15 +2438,15 @@
         <v>0.70000000000000007</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -2445,15 +2459,15 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="F67" s="5" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="11" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C68">
         <v>1</v>
@@ -2466,15 +2480,15 @@
         <v>0.11</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C69">
         <v>4</v>
@@ -2492,10 +2506,10 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -2513,10 +2527,10 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -2529,15 +2543,15 @@
         <v>0.12</v>
       </c>
       <c r="F71" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="72" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C72">
         <v>10</v>
@@ -2550,15 +2564,15 @@
         <v>1.7999999999999998</v>
       </c>
       <c r="F72" s="5" t="s">
-        <v>109</v>
+        <v>316</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="11" t="s">
-        <v>95</v>
+        <v>319</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C73">
         <v>1</v>
@@ -2571,15 +2585,15 @@
         <v>0.76</v>
       </c>
       <c r="F73" s="5" t="s">
-        <v>162</v>
+        <v>318</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C74">
         <v>1</v>
@@ -2592,15 +2606,15 @@
         <v>0.89</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="75" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B75" s="7" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C75">
         <v>1</v>
@@ -2613,20 +2627,20 @@
         <v>0.99</v>
       </c>
       <c r="F75" s="5" t="s">
-        <v>115</v>
+        <v>317</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B78" s="7" t="s">
         <v>78</v>
-      </c>
-      <c r="B78" s="7" t="s">
-        <v>79</v>
       </c>
       <c r="C78">
         <v>1</v>
@@ -2644,10 +2658,10 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="B79" s="7" t="s">
-        <v>83</v>
       </c>
       <c r="C79">
         <v>1</v>
@@ -2665,10 +2679,10 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B80" s="7" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C80">
         <v>1</v>
@@ -2681,7 +2695,7 @@
         <v>0.37</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -2692,13 +2706,13 @@
         <v>3</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D82" s="3"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B83" s="9">
         <f>SUM(E2:E80)</f>
@@ -2748,36 +2762,42 @@
     <hyperlink ref="F50" r:id="rId17" xr:uid="{27AFE47D-7B3E-4AD0-9835-34F6B55F8FF0}"/>
     <hyperlink ref="F54" r:id="rId18" xr:uid="{B166CAA7-8FF4-4B71-ABC8-56AF926B1EE3}"/>
     <hyperlink ref="F55" r:id="rId19" xr:uid="{E4FC7202-360B-49B9-BE38-D63B47270DAE}"/>
-    <hyperlink ref="F72" r:id="rId20" xr:uid="{E12BC84C-E61B-43B0-AE1B-CC7D351CF365}"/>
-    <hyperlink ref="F70" r:id="rId21" xr:uid="{C22CD521-6043-45A6-8FDB-24E605523556}"/>
-    <hyperlink ref="F21" r:id="rId22" xr:uid="{A877581D-DAE2-49DF-AFDF-7BDA2C30D7E6}"/>
-    <hyperlink ref="F75" r:id="rId23" xr:uid="{3D243AA0-BEF7-4408-A77A-97FD51037221}"/>
-    <hyperlink ref="F17" r:id="rId24" xr:uid="{5563CFDB-A3BC-4AE4-8718-0948D1325788}"/>
-    <hyperlink ref="F36" r:id="rId25" xr:uid="{A52F5B26-597E-4DC3-8C15-3B2876C00684}"/>
-    <hyperlink ref="F59" r:id="rId26" xr:uid="{EE5FB14A-DB2C-404D-9BDD-DBCC5B795F87}"/>
-    <hyperlink ref="F62" r:id="rId27" xr:uid="{AC0283C7-85A9-414F-9521-28C6E8D6C24D}"/>
-    <hyperlink ref="F5" r:id="rId28" xr:uid="{C0D297E1-764F-4191-9557-3C0BB3DA76E0}"/>
-    <hyperlink ref="F80" r:id="rId29" xr:uid="{AEE228DF-40B3-4EDE-AE80-DBFD429B606F}"/>
-    <hyperlink ref="F24" r:id="rId30" xr:uid="{7C7F06CF-3B10-4DFA-972A-6E4E4223480E}"/>
-    <hyperlink ref="F4" r:id="rId31" xr:uid="{381D13AF-9DB9-48A4-A212-31B4F89C8051}"/>
-    <hyperlink ref="F73" r:id="rId32" display="https://www.digikey.com/en/products/detail/avx-corporation/F980J107MMAAXE/5957626?s=N4IgjCBcpgbFoDGUBmBDANgZwKYBoQB7KAbRAGYBOAJgBZ4BdAgBwBcoQBlVgJwEsAdgHMQAXwJhKADkoIQySOmz4ipEAAYQTEGw7d%2BwsQWrras6DvaQQAVQF9WAeRQBZHGiwBXHjhAFPHACtAGJ%2BIAC2ghxg6poE4WgAHtGxRiAmAOzmSKiYuATEkGSwAGphsAB05GUEUjXg6vVgAKxNpWEm9dStYeSNvT0EtP0EzSMgsONg3WXautZ2Ds5uHt6%2BouLpaohozGiIDoQ8WqJAA" xr:uid="{EABCF24D-2C02-411B-B75C-2324775E94EE}"/>
-    <hyperlink ref="F66" r:id="rId33" xr:uid="{483529F7-C4C0-4B52-BB5C-60E6A3188AF6}"/>
-    <hyperlink ref="F74" r:id="rId34" xr:uid="{C919FD41-64A3-49E2-8D89-9FA957D6C873}"/>
-    <hyperlink ref="F18" r:id="rId35" xr:uid="{66DC527E-1B36-4735-94CD-9D37A6062B3A}"/>
-    <hyperlink ref="F65" r:id="rId36" xr:uid="{C8962D43-B0E0-4EC5-B4C6-EF2A9B9C4FA6}"/>
-    <hyperlink ref="F68" r:id="rId37" xr:uid="{40EA68E7-CC0F-402F-BD34-38FB90FF4C83}"/>
-    <hyperlink ref="F49" r:id="rId38" xr:uid="{FC1E67BF-EAA3-45A1-8AF2-6FC11BAD1CAB}"/>
-    <hyperlink ref="F56" r:id="rId39" xr:uid="{CF4C28CD-42DB-410E-93A8-2CA1C27A8C6A}"/>
-    <hyperlink ref="F6" r:id="rId40" xr:uid="{88B43D37-ED21-421E-8DE4-4A9BC1856308}"/>
-    <hyperlink ref="F32" r:id="rId41" xr:uid="{A168D9F0-C6CE-4665-8C5B-EB1FF16812E5}"/>
-    <hyperlink ref="F7" r:id="rId42" xr:uid="{5A545753-6BAE-4E93-BD3F-7015D416345E}"/>
-    <hyperlink ref="F8" r:id="rId43" xr:uid="{1D57C2C6-69F9-44B1-964A-8806C8F505BE}"/>
-    <hyperlink ref="F9" r:id="rId44" xr:uid="{0FF96674-38C4-43D9-8178-B8612EF4B766}"/>
-    <hyperlink ref="F10" r:id="rId45" xr:uid="{240C0BBB-5F46-443B-8975-6A4001EE6F2C}"/>
-    <hyperlink ref="F11" r:id="rId46" xr:uid="{AD6D1C95-A83C-44FC-B812-7856EDE97CD8}"/>
+    <hyperlink ref="F70" r:id="rId20" xr:uid="{C22CD521-6043-45A6-8FDB-24E605523556}"/>
+    <hyperlink ref="F21" r:id="rId21" xr:uid="{A877581D-DAE2-49DF-AFDF-7BDA2C30D7E6}"/>
+    <hyperlink ref="F17" r:id="rId22" xr:uid="{5563CFDB-A3BC-4AE4-8718-0948D1325788}"/>
+    <hyperlink ref="F36" r:id="rId23" xr:uid="{A52F5B26-597E-4DC3-8C15-3B2876C00684}"/>
+    <hyperlink ref="F59" r:id="rId24" xr:uid="{EE5FB14A-DB2C-404D-9BDD-DBCC5B795F87}"/>
+    <hyperlink ref="F62" r:id="rId25" xr:uid="{AC0283C7-85A9-414F-9521-28C6E8D6C24D}"/>
+    <hyperlink ref="F5" r:id="rId26" xr:uid="{C0D297E1-764F-4191-9557-3C0BB3DA76E0}"/>
+    <hyperlink ref="F80" r:id="rId27" xr:uid="{AEE228DF-40B3-4EDE-AE80-DBFD429B606F}"/>
+    <hyperlink ref="F24" r:id="rId28" xr:uid="{7C7F06CF-3B10-4DFA-972A-6E4E4223480E}"/>
+    <hyperlink ref="F4" r:id="rId29" xr:uid="{381D13AF-9DB9-48A4-A212-31B4F89C8051}"/>
+    <hyperlink ref="F66" r:id="rId30" xr:uid="{483529F7-C4C0-4B52-BB5C-60E6A3188AF6}"/>
+    <hyperlink ref="F74" r:id="rId31" xr:uid="{C919FD41-64A3-49E2-8D89-9FA957D6C873}"/>
+    <hyperlink ref="F18" r:id="rId32" xr:uid="{66DC527E-1B36-4735-94CD-9D37A6062B3A}"/>
+    <hyperlink ref="F65" r:id="rId33" xr:uid="{C8962D43-B0E0-4EC5-B4C6-EF2A9B9C4FA6}"/>
+    <hyperlink ref="F68" r:id="rId34" xr:uid="{40EA68E7-CC0F-402F-BD34-38FB90FF4C83}"/>
+    <hyperlink ref="F49" r:id="rId35" xr:uid="{FC1E67BF-EAA3-45A1-8AF2-6FC11BAD1CAB}"/>
+    <hyperlink ref="F56" r:id="rId36" xr:uid="{CF4C28CD-42DB-410E-93A8-2CA1C27A8C6A}"/>
+    <hyperlink ref="F6" r:id="rId37" xr:uid="{88B43D37-ED21-421E-8DE4-4A9BC1856308}"/>
+    <hyperlink ref="F32" r:id="rId38" xr:uid="{A168D9F0-C6CE-4665-8C5B-EB1FF16812E5}"/>
+    <hyperlink ref="F7" r:id="rId39" xr:uid="{5A545753-6BAE-4E93-BD3F-7015D416345E}"/>
+    <hyperlink ref="F8" r:id="rId40" xr:uid="{1D57C2C6-69F9-44B1-964A-8806C8F505BE}"/>
+    <hyperlink ref="F9" r:id="rId41" xr:uid="{0FF96674-38C4-43D9-8178-B8612EF4B766}"/>
+    <hyperlink ref="F10" r:id="rId42" xr:uid="{240C0BBB-5F46-443B-8975-6A4001EE6F2C}"/>
+    <hyperlink ref="F11" r:id="rId43" xr:uid="{AD6D1C95-A83C-44FC-B812-7856EDE97CD8}"/>
+    <hyperlink ref="F28" r:id="rId44" xr:uid="{2078B4D5-94F7-4DF6-8342-B722D4BA5A8B}"/>
+    <hyperlink ref="F29" r:id="rId45" xr:uid="{85BE8015-0AC5-408F-A118-D71CE05A8A73}"/>
+    <hyperlink ref="F40" r:id="rId46" xr:uid="{2D77AB52-9F3A-475F-BC04-828C40F93148}"/>
+    <hyperlink ref="F57" r:id="rId47" xr:uid="{13386EBC-64DC-4E8C-A7B2-3489A8FDDFBC}"/>
+    <hyperlink ref="F63" r:id="rId48" xr:uid="{445B1E67-E918-4933-BFC4-6DD1B3DE410B}"/>
+    <hyperlink ref="F64" r:id="rId49" xr:uid="{5DB93F23-2C28-4696-90F8-B2A33BFED473}"/>
+    <hyperlink ref="F67" r:id="rId50" xr:uid="{11B0603D-FFC6-4208-AAB2-F094CB915B81}"/>
+    <hyperlink ref="F71" r:id="rId51" xr:uid="{52AB4B2E-A871-4BD0-A4F3-CDA900B05973}"/>
+    <hyperlink ref="F72" r:id="rId52" xr:uid="{D0F23DDA-D9F1-45BE-998F-A171C0A640F7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId47"/>
+  <pageSetup orientation="portrait" r:id="rId53"/>
 </worksheet>
 </file>
 
@@ -2797,7 +2817,7 @@
         <v>21</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -2814,37 +2834,37 @@
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B2" s="8"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>248</v>
+        <v>313</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" s="4">
-        <v>1.17</v>
+        <v>6.41</v>
       </c>
       <c r="E3" s="4">
         <f>D3*C3</f>
-        <v>1.17</v>
+        <v>6.41</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>34</v>
+        <v>314</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -2857,15 +2877,15 @@
         <v>2.5099999999999998</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -2878,7 +2898,7 @@
         <v>0.91</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -2886,16 +2906,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="B7" s="8"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B8" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -2908,15 +2928,15 @@
         <v>0.68</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -2929,15 +2949,15 @@
         <v>2.92</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -2950,15 +2970,15 @@
         <v>1.75</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -2971,15 +2991,15 @@
         <v>0.39</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -2992,7 +3012,7 @@
         <v>0.39</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -3000,28 +3020,28 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15" s="4">
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="E15" s="4">
         <f>D15*C15</f>
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>268</v>
+        <v>311</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -3038,7 +3058,7 @@
         <v>6</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C18">
         <v>4</v>
@@ -3056,37 +3076,37 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
       <c r="D19" s="4">
-        <v>1.7</v>
+        <v>6.7</v>
       </c>
       <c r="E19" s="4">
         <f>D19*C19</f>
-        <v>1.7</v>
+        <v>6.7</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>275</v>
+        <v>315</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B21" s="8"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -3099,15 +3119,15 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -3120,7 +3140,7 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -3128,16 +3148,16 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B25" s="8"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -3150,7 +3170,7 @@
         <v>0.42</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -3158,7 +3178,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B28" s="8"/>
       <c r="F28" s="5"/>
@@ -3168,7 +3188,7 @@
         <v>16</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -3190,17 +3210,17 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B31" s="1"/>
       <c r="F31" s="5"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -3213,15 +3233,15 @@
         <v>0.1</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="C33">
         <v>2</v>
@@ -3234,15 +3254,15 @@
         <v>0.36</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -3255,15 +3275,15 @@
         <v>0.1</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="C35">
         <v>10</v>
@@ -3281,10 +3301,10 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -3297,15 +3317,15 @@
         <v>0.22</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="C37">
         <v>2</v>
@@ -3318,7 +3338,7 @@
         <v>0.2</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -3328,17 +3348,17 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B39" s="1"/>
       <c r="F39" s="5"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C40">
         <v>2</v>
@@ -3351,15 +3371,15 @@
         <v>0.4</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="C41">
         <v>6</v>
@@ -3372,15 +3392,15 @@
         <v>0.60000000000000009</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="C42">
         <v>11</v>
@@ -3398,10 +3418,10 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -3419,10 +3439,10 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="C44">
         <v>5</v>
@@ -3435,15 +3455,15 @@
         <v>0.89999999999999991</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="C45">
         <v>2</v>
@@ -3456,20 +3476,20 @@
         <v>0.96</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="C48">
         <v>2</v>
@@ -3482,7 +3502,7 @@
         <v>0.2</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -3490,21 +3510,21 @@
         <v>3</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D50" s="3"/>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B51" s="9">
         <f>SUM(E2:E49)</f>
-        <v>25.240000000000002</v>
+        <v>35.500000000000007</v>
       </c>
       <c r="C51" s="4">
         <f>B51/1</f>
-        <v>25.240000000000002</v>
+        <v>35.500000000000007</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -3538,20 +3558,23 @@
     <hyperlink ref="F43" r:id="rId9" xr:uid="{266C3A64-556B-4754-A0CA-60FAB18F6801}"/>
     <hyperlink ref="F45" r:id="rId10" xr:uid="{4C8275B9-6378-4194-B04A-9249EF2C3F3B}"/>
     <hyperlink ref="F32" r:id="rId11" xr:uid="{350463DE-E3C0-449B-8091-96279D64BDA7}"/>
-    <hyperlink ref="F3" r:id="rId12" xr:uid="{8C6F62A0-0E77-4E68-9138-404EE92E4AE4}"/>
-    <hyperlink ref="F4" r:id="rId13" xr:uid="{BB561A52-3DD9-4A70-AF7E-2618E9200F2E}"/>
-    <hyperlink ref="F18" r:id="rId14" xr:uid="{3A57A089-47DB-4C5B-8942-DEFD8232EFEE}"/>
-    <hyperlink ref="F23" r:id="rId15" xr:uid="{683E87C4-72FD-4154-A63F-ACE4F30B290A}"/>
-    <hyperlink ref="F22" r:id="rId16" xr:uid="{A961D329-A7D1-44CF-9871-E72A5B53CFB7}"/>
-    <hyperlink ref="F10" r:id="rId17" xr:uid="{A571335B-00BC-4DD5-BF5B-8CB442E891E0}"/>
-    <hyperlink ref="F15" r:id="rId18" xr:uid="{1B92BE63-5213-40E7-8D62-B3E0E067C5BF}"/>
-    <hyperlink ref="F35" r:id="rId19" xr:uid="{0FF516AE-C3FF-4485-9872-2719916BD263}"/>
-    <hyperlink ref="F34" r:id="rId20" xr:uid="{311BC1A4-1213-4AD6-93EB-15BA831AC69A}"/>
-    <hyperlink ref="F41" r:id="rId21" xr:uid="{469E9AFB-BF8A-49CD-8753-62E512A8B747}"/>
-    <hyperlink ref="F19" r:id="rId22" display="https://www.ebay.com/itm/354618455099?chn=ps&amp;var=623990696410&amp;_trkparms=ispr%3D1&amp;amdata=enc%3A1Zk6c1fiYQTmjnu1i-GLg_w51&amp;norover=1&amp;mkevt=1&amp;mkrid=711-117182-37290-0&amp;mkcid=2&amp;mkscid=101&amp;itemid=623990696410_354618455099&amp;targetid=1584739238534&amp;device=c&amp;mktype=&amp;googleloc=9016965&amp;poi=&amp;campaignid=15275224983&amp;mkgroupid=131097072938&amp;rlsatarget=pla-1584739238534&amp;abcId=9300697&amp;merchantid=633191918&amp;gclid=CjwKCAjw3ueiBhBmEiwA4BhspPro6b1IzauVdwTaQfRWhvR-m2RbObJTIP_17MVH22aw1EJwAAuf9hoCW1kQAvD_BwE" xr:uid="{FFB58D04-F635-4E08-965C-1F1978413F1B}"/>
+    <hyperlink ref="F4" r:id="rId12" xr:uid="{BB561A52-3DD9-4A70-AF7E-2618E9200F2E}"/>
+    <hyperlink ref="F18" r:id="rId13" xr:uid="{3A57A089-47DB-4C5B-8942-DEFD8232EFEE}"/>
+    <hyperlink ref="F23" r:id="rId14" xr:uid="{683E87C4-72FD-4154-A63F-ACE4F30B290A}"/>
+    <hyperlink ref="F22" r:id="rId15" xr:uid="{A961D329-A7D1-44CF-9871-E72A5B53CFB7}"/>
+    <hyperlink ref="F10" r:id="rId16" xr:uid="{A571335B-00BC-4DD5-BF5B-8CB442E891E0}"/>
+    <hyperlink ref="F35" r:id="rId17" xr:uid="{0FF516AE-C3FF-4485-9872-2719916BD263}"/>
+    <hyperlink ref="F34" r:id="rId18" xr:uid="{311BC1A4-1213-4AD6-93EB-15BA831AC69A}"/>
+    <hyperlink ref="F41" r:id="rId19" xr:uid="{469E9AFB-BF8A-49CD-8753-62E512A8B747}"/>
+    <hyperlink ref="F5" r:id="rId20" xr:uid="{EB58DEF7-4869-4B45-9862-8732A0709EA7}"/>
+    <hyperlink ref="F8" r:id="rId21" xr:uid="{372FDDE4-4024-4EE9-8648-17195775C560}"/>
+    <hyperlink ref="F9" r:id="rId22" xr:uid="{3AA4E8B5-3892-4787-85CD-6CCCD2D10F9F}"/>
+    <hyperlink ref="F11" r:id="rId23" xr:uid="{5333A484-C9E0-44B3-B945-42F28906F373}"/>
+    <hyperlink ref="F12" r:id="rId24" xr:uid="{1F3F49F8-9803-409E-A9D1-5774B1E9124E}"/>
+    <hyperlink ref="F40" r:id="rId25" xr:uid="{2412A0E1-8EF9-418C-ACB9-6A973D420171}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId23"/>
+  <pageSetup orientation="portrait" r:id="rId26"/>
 </worksheet>
 </file>
 
@@ -3571,7 +3594,7 @@
         <v>21</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -3588,16 +3611,16 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="B2" s="8"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B3" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -3610,15 +3633,15 @@
         <v>0.68</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -3631,15 +3654,15 @@
         <v>1.75</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -3652,15 +3675,15 @@
         <v>0.39</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -3673,7 +3696,7 @@
         <v>0.39</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -3681,28 +3704,28 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" s="4">
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="E9" s="4">
         <f>D9*C9</f>
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>268</v>
+        <v>311</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -3716,37 +3739,37 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" s="4">
-        <v>1.7</v>
+        <v>6.5</v>
       </c>
       <c r="E12" s="4">
         <f>D12*C12</f>
-        <v>1.7</v>
+        <v>6.5</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>275</v>
+        <v>312</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B14" s="8"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -3759,15 +3782,15 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -3780,7 +3803,7 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -3788,16 +3811,16 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B18" s="8"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -3810,7 +3833,7 @@
         <v>0.42</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -3818,7 +3841,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B21" s="8"/>
       <c r="F21" s="5"/>
@@ -3828,7 +3851,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -3850,17 +3873,17 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B24" s="1"/>
       <c r="F24" s="5"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -3873,15 +3896,15 @@
         <v>0.1</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -3904,17 +3927,17 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B28" s="1"/>
       <c r="F28" s="5"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C29">
         <v>2</v>
@@ -3927,15 +3950,15 @@
         <v>0.2</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -3948,7 +3971,7 @@
         <v>0.18</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -3956,21 +3979,21 @@
         <v>3</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D32" s="3"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B33" s="9">
         <f>SUM(E2:E31)</f>
-        <v>7.29</v>
+        <v>12.11</v>
       </c>
       <c r="C33" s="4">
         <f>B33/1</f>
-        <v>7.29</v>
+        <v>12.11</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -3999,10 +4022,12 @@
     <hyperlink ref="F16" r:id="rId4" xr:uid="{08EA6188-8D92-45D6-9FB1-75D44E2F4E17}"/>
     <hyperlink ref="F15" r:id="rId5" xr:uid="{0990DBEB-9B40-4154-B935-D0AE3765815B}"/>
     <hyperlink ref="F4" r:id="rId6" xr:uid="{3A6A8E0D-8272-4082-B333-B3E51994AB11}"/>
-    <hyperlink ref="F9" r:id="rId7" xr:uid="{4F32BAC5-E459-4D66-A782-992CFD41EB9D}"/>
-    <hyperlink ref="F26" r:id="rId8" xr:uid="{C3148856-4EEB-48B9-A415-3F9D97E01223}"/>
-    <hyperlink ref="F25" r:id="rId9" xr:uid="{53D54B38-4438-4D1D-BCDC-B9CC580A2AAF}"/>
-    <hyperlink ref="F29" r:id="rId10" xr:uid="{7421347A-AD22-4C92-8F37-14B7A9DCFBED}"/>
+    <hyperlink ref="F26" r:id="rId7" xr:uid="{C3148856-4EEB-48B9-A415-3F9D97E01223}"/>
+    <hyperlink ref="F25" r:id="rId8" xr:uid="{53D54B38-4438-4D1D-BCDC-B9CC580A2AAF}"/>
+    <hyperlink ref="F29" r:id="rId9" xr:uid="{7421347A-AD22-4C92-8F37-14B7A9DCFBED}"/>
+    <hyperlink ref="F3" r:id="rId10" xr:uid="{F982D18A-A48F-4C43-808F-8BBFD0A85C3A}"/>
+    <hyperlink ref="F5" r:id="rId11" xr:uid="{BC20A03D-6D23-4AD5-A4BC-E35099B8E7F7}"/>
+    <hyperlink ref="F6" r:id="rId12" xr:uid="{2A3C64B8-6EB5-495D-A04E-0F5EFECF676C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4017,7 +4042,9 @@
     <col min="2" max="2" width="20" style="4" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" customWidth="1"/>
     <col min="4" max="4" width="11.5703125" style="4" customWidth="1"/>
-    <col min="5" max="8" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" customWidth="1"/>
+    <col min="6" max="6" width="61.28515625" customWidth="1"/>
+    <col min="7" max="8" width="11.5703125" customWidth="1"/>
     <col min="9" max="9" width="128.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4040,10 +4067,10 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -4061,23 +4088,23 @@
     </row>
     <row r="3" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" s="4">
-        <v>9.99</v>
+        <v>10.81</v>
       </c>
       <c r="E3" s="4">
         <f t="shared" ref="E3:E10" si="0">D3*C3</f>
-        <v>9.99</v>
+        <v>10.81</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -4085,7 +4112,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -4098,7 +4125,7 @@
         <v>7.94</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -4106,28 +4133,28 @@
         <v>10</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" s="4">
-        <v>12.95</v>
+        <v>27</v>
       </c>
       <c r="E5" s="4">
         <f>D5*C5</f>
-        <v>12.95</v>
+        <v>27</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>242</v>
+        <v>308</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -4140,7 +4167,7 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -4148,29 +4175,29 @@
         <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" s="4">
-        <v>9.6199999999999992</v>
+        <v>13.5</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="0"/>
-        <v>9.6199999999999992</v>
+        <v>13.5</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="G7" s="7"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -4183,15 +4210,15 @@
         <v>8.69</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -4204,15 +4231,15 @@
         <v>4.34</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -4225,7 +4252,7 @@
         <v>0.47</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -4233,7 +4260,7 @@
         <v>31</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -4251,31 +4278,31 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" s="4">
-        <v>24.76</v>
+        <v>40.03</v>
       </c>
       <c r="E12" s="4">
         <f t="shared" si="1"/>
-        <v>24.76</v>
+        <v>40.03</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -4288,15 +4315,15 @@
         <v>1.93</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -4309,15 +4336,15 @@
         <v>1.86</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -4330,15 +4357,15 @@
         <v>13.28</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -4351,7 +4378,7 @@
         <v>13.99</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -4361,17 +4388,17 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="B18" s="7"/>
       <c r="E18" s="4"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -4384,15 +4411,15 @@
         <v>2.68</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="C20">
         <v>4</v>
@@ -4405,7 +4432,7 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -4415,14 +4442,14 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B22" s="7"/>
       <c r="E22" s="10"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B23" s="7"/>
       <c r="D23">
@@ -4432,7 +4459,7 @@
         <v>6.9</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -4444,7 +4471,7 @@
       </c>
       <c r="E25" s="4">
         <f>SUM(E2:E23)</f>
-        <v>177.16000000000003</v>
+        <v>211.18000000000004</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -4456,12 +4483,16 @@
       <c r="E27" s="5"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="2"/>
+      <c r="A28" s="16" t="s">
+        <v>309</v>
+      </c>
       <c r="B28" s="2"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
+      <c r="F28" s="15" t="s">
+        <v>310</v>
+      </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="2"/>
@@ -4668,10 +4699,16 @@
     <hyperlink ref="F10" r:id="rId6" xr:uid="{C96AEF29-4AC2-4257-8AB3-AE09B73FA388}"/>
     <hyperlink ref="F19" r:id="rId7" xr:uid="{85344F48-5909-4D4E-82AA-60C131CCB21A}"/>
     <hyperlink ref="F8" r:id="rId8" display="https://www.amazon.com/Dedicated-Aluminum-Heatsink-Raspberry-Compute/dp/B093FSS6XX/ref=asc_df_B093FSS6XX/?tag=hyprod-20&amp;linkCode=df0&amp;hvadid=647248209079&amp;hvpos=&amp;hvnetw=g&amp;hvrand=4581538439163296605&amp;hvpone=&amp;hvptwo=&amp;hvqmt=&amp;hvdev=c&amp;hvdvcmdl=&amp;hvlocint=&amp;hvlocphy=9016965&amp;hvtargid=pla-2007964195647&amp;gclid=CjwKCAjw3ueiBhBmEiwA4BhspC4oXb-6Z3YZKl8dphxldkEmSZ_R6mIv_rni8NS5jTlwWlrca2spgRoCp7AQAvD_BwE&amp;th=1" xr:uid="{4D06C1FE-87B7-4C95-A120-D58694B9DB38}"/>
-    <hyperlink ref="F7" r:id="rId9" display="https://www.aliexpress.us/item/3256803228333750.html?spm=a2g0o.productlist.main.1.27357aedfOveIi&amp;algo_pvid=b9289e00-9e59-4056-b51a-43910fcea86f&amp;algo_exp_id=b9289e00-9e59-4056-b51a-43910fcea86f-0&amp;pdp_npi=3%40dis%21USD%2111.59%219.62%21%21%21%21%21%40212278bd16865808440348119d07cd%2112000025683190881%21sea%21US%211888726260&amp;curPageLogUid=DbxWuEx0YQy9" xr:uid="{5CC8DA23-2F67-4CD0-A0DF-630E6A932E55}"/>
+    <hyperlink ref="F28" r:id="rId9" xr:uid="{EB55229C-F54B-4C46-94E1-24EE1011AE7A}"/>
+    <hyperlink ref="F9" r:id="rId10" xr:uid="{51B52101-2A4A-4111-9EB0-D94FF7DAF0BF}"/>
+    <hyperlink ref="F13" r:id="rId11" xr:uid="{5D17CDAE-E94A-464E-BDBE-4D010517E3BC}"/>
+    <hyperlink ref="F14" r:id="rId12" xr:uid="{556B9FF1-B5FF-4C94-B027-5745DB6A4DC2}"/>
+    <hyperlink ref="F15" r:id="rId13" display="https://www.ebay.com/itm/174968443925?_trkparms=amclksrc%3DITM%26aid%3D777008%26algo%3DPERSONAL.TOPIC%26ao%3D1%26asc%3D20220705100511%26meid%3D2faa5f1c66e54ff3af69f69cbfe6d567%26pid%3D101524%26rk%3D1%26rkt%3D1%26itm%3D174968443925%26pmt%3D1%26noa%3D1%26pg%3D2380057%26algv%3DRecentlyViewedItemsV2&amp;_trksid=p2380057.c101524.m146925&amp;_trkparms=pageci%3Aca4f6cab-ee8f-11ed-9b33-d2bafba4db3b%7Cparentrq%3A019472791880a69e559fc3aafffefea4%7Ciid%3A1" xr:uid="{24EF6E9B-3278-49A3-92E9-C39691B78F2E}"/>
+    <hyperlink ref="F16" r:id="rId14" xr:uid="{1078468C-9681-4B8B-B881-6DF6F32C87FA}"/>
+    <hyperlink ref="F20" r:id="rId15" xr:uid="{A4B0540A-680F-4F3A-A223-E547C41E6857}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId10"/>
+  <pageSetup orientation="portrait" r:id="rId16"/>
 </worksheet>
 </file>
 
@@ -4705,7 +4742,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -4718,7 +4755,7 @@
         <v>15.99</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -4736,12 +4773,12 @@
         <v>12.99</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -4754,12 +4791,12 @@
         <v>8.99</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -4772,7 +4809,7 @@
         <v>6.9</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -4938,6 +4975,12 @@
       <c r="A72" s="5"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{C3C1328F-63D7-4691-A4B3-E21DC5778032}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{645A7889-B381-4182-855B-534A6345470E}"/>
+    <hyperlink ref="E4" r:id="rId3" xr:uid="{E30ECB10-46ED-44E3-8C43-A1B31DFCEE74}"/>
+    <hyperlink ref="E5" r:id="rId4" xr:uid="{E7E82358-E3A0-41DA-9E71-9FDFCE8B4D7B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: added the clear acrylic sheet to the BOM for the front of the screen
</commit_message>
<xml_diff>
--- a/Version WIP/Aegis 2 BOM.xlsx
+++ b/Version WIP/Aegis 2 BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jucke\Dropbox\Projects\Aegis 2\Aegis-2\Version WIP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D29D3D4B-318A-4E78-ABDD-27C0D878FA11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06BB469-A0B9-44F0-ABEF-896FEEA4D6FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{93BD1906-D6D6-45EE-A20C-B1437B097662}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{93BD1906-D6D6-45EE-A20C-B1437B097662}"/>
   </bookViews>
   <sheets>
     <sheet name="Main Board" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="323">
   <si>
     <t>Qty</t>
   </si>
@@ -997,6 +997,15 @@
   </si>
   <si>
     <t>Cap 100uF (805)</t>
+  </si>
+  <si>
+    <t>ACRYLIC</t>
+  </si>
+  <si>
+    <t>Clear Acrylic Custom Size (6.5" x 4.125" x 1mm)</t>
+  </si>
+  <si>
+    <t>https://www.canalplastic.com/products/clear-colorless-0-040-acrylic-sheet?variant=37615076302</t>
   </si>
 </sst>
 </file>
@@ -1079,7 +1088,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1112,7 +1121,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4035,7 +4043,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9192E0A5-2D05-4B52-937A-084865A72460}">
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.42578125" customWidth="1"/>
@@ -4269,7 +4277,7 @@
         <v>40</v>
       </c>
       <c r="E11" s="4">
-        <f t="shared" ref="E11:E16" si="1">D11*C11</f>
+        <f t="shared" ref="E11:E17" si="1">D11*C11</f>
         <v>40</v>
       </c>
       <c r="F11" s="5" t="s">
@@ -4382,130 +4390,141 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B17" s="7"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="5"/>
+      <c r="A17" t="s">
+        <v>321</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4">
+        <v>3.9</v>
+      </c>
+      <c r="E17" s="4">
+        <f t="shared" si="1"/>
+        <v>3.9</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>256</v>
-      </c>
       <c r="B18" s="7"/>
       <c r="E18" s="4"/>
+      <c r="F18" s="5"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>251</v>
-      </c>
-      <c r="B19" s="7" t="s">
-        <v>252</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-      <c r="D19" s="4">
-        <v>2.68</v>
-      </c>
-      <c r="E19" s="4">
-        <f>D19*C19</f>
-        <v>2.68</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>263</v>
-      </c>
+      <c r="A19" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B19" s="7"/>
+      <c r="E19" s="4"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="C20">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D20" s="4">
-        <v>2.2999999999999998</v>
+        <v>2.68</v>
       </c>
       <c r="E20" s="4">
         <f>D20*C20</f>
+        <v>2.68</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>258</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="C21">
+        <v>4</v>
+      </c>
+      <c r="D21" s="4">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E21" s="4">
+        <f>D21*C21</f>
         <v>9.1999999999999993</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F21" s="5" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B21" s="7"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="5"/>
-    </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="B22" s="7"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B22" s="7"/>
-      <c r="E22" s="10"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="B23" s="7"/>
+      <c r="E23" s="10"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>116</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="E23" s="10">
+      <c r="B24" s="7"/>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24" s="10">
         <v>6.9</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F24" s="5" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E24" s="5"/>
-    </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+      <c r="E25" s="5"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E25" s="4">
-        <f>SUM(E2:E23)</f>
-        <v>211.18000000000004</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="6"/>
-      <c r="E26" s="5"/>
+      <c r="E26" s="4">
+        <f>SUM(E2:E24)</f>
+        <v>215.08000000000004</v>
+      </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="E27" s="5"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="6"/>
+      <c r="E28" s="5"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>309</v>
       </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="15" t="s">
+      <c r="B29" s="2"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="15" t="s">
         <v>310</v>
       </c>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="2"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B29" s="7"/>
-      <c r="C29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="2"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B30" s="7"/>
@@ -4514,6 +4533,8 @@
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B31" s="7"/>
@@ -4548,9 +4569,12 @@
       <c r="H34" s="4"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="2"/>
       <c r="B35" s="7"/>
-      <c r="E35" s="5"/>
+      <c r="C35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
@@ -4558,14 +4582,13 @@
       <c r="E36" s="5"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B37" s="8"/>
-      <c r="C37" s="2"/>
+      <c r="A37" s="2"/>
+      <c r="B37" s="7"/>
       <c r="E37" s="5"/>
     </row>
-    <row r="38" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="2"/>
-      <c r="B38" s="9"/>
-      <c r="C38" s="4"/>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B38" s="8"/>
+      <c r="C38" s="2"/>
       <c r="E38" s="5"/>
     </row>
     <row r="39" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4574,13 +4597,16 @@
       <c r="C39" s="4"/>
       <c r="E39" s="5"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="9"/>
       <c r="C40" s="4"/>
       <c r="E40" s="5"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="2"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="4"/>
       <c r="E41" s="5"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -4619,14 +4645,14 @@
     <row r="53" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E53" s="5"/>
     </row>
-    <row r="54" spans="5:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E54" s="5"/>
     </row>
     <row r="55" spans="5:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E55" s="5"/>
     </row>
-    <row r="57" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E57" s="5"/>
+    <row r="56" spans="5:5" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E56" s="5"/>
     </row>
     <row r="58" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E58" s="5"/>
@@ -4659,35 +4685,38 @@
       <c r="E67" s="5"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="2"/>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="2"/>
+      <c r="E68" s="5"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="2"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="1"/>
-      <c r="E72" s="5"/>
+      <c r="A72" s="2"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="6"/>
+      <c r="A73" s="1"/>
       <c r="E73" s="5"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="6"/>
       <c r="E74" s="5"/>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="2"/>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="6"/>
+      <c r="E75" s="5"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="E88" s="5"/>
+      <c r="A88" s="2"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E89" s="5"/>
     </row>
-    <row r="94" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="5"/>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E90" s="5"/>
+    </row>
+    <row r="95" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" s="5"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -4695,17 +4724,17 @@
     <hyperlink ref="F6" r:id="rId2" xr:uid="{67359FE7-E187-4642-A73D-A178EF9B7A83}"/>
     <hyperlink ref="F4" r:id="rId3" xr:uid="{5DF653D7-A7D4-462D-B589-02D1118DB8DB}"/>
     <hyperlink ref="F2" r:id="rId4" xr:uid="{84970AA0-897C-43E7-B8DF-28D3F3300098}"/>
-    <hyperlink ref="F23" r:id="rId5" xr:uid="{216EE6A3-8045-4544-8D98-ABDA82CD9234}"/>
+    <hyperlink ref="F24" r:id="rId5" xr:uid="{216EE6A3-8045-4544-8D98-ABDA82CD9234}"/>
     <hyperlink ref="F10" r:id="rId6" xr:uid="{C96AEF29-4AC2-4257-8AB3-AE09B73FA388}"/>
-    <hyperlink ref="F19" r:id="rId7" xr:uid="{85344F48-5909-4D4E-82AA-60C131CCB21A}"/>
+    <hyperlink ref="F20" r:id="rId7" xr:uid="{85344F48-5909-4D4E-82AA-60C131CCB21A}"/>
     <hyperlink ref="F8" r:id="rId8" display="https://www.amazon.com/Dedicated-Aluminum-Heatsink-Raspberry-Compute/dp/B093FSS6XX/ref=asc_df_B093FSS6XX/?tag=hyprod-20&amp;linkCode=df0&amp;hvadid=647248209079&amp;hvpos=&amp;hvnetw=g&amp;hvrand=4581538439163296605&amp;hvpone=&amp;hvptwo=&amp;hvqmt=&amp;hvdev=c&amp;hvdvcmdl=&amp;hvlocint=&amp;hvlocphy=9016965&amp;hvtargid=pla-2007964195647&amp;gclid=CjwKCAjw3ueiBhBmEiwA4BhspC4oXb-6Z3YZKl8dphxldkEmSZ_R6mIv_rni8NS5jTlwWlrca2spgRoCp7AQAvD_BwE&amp;th=1" xr:uid="{4D06C1FE-87B7-4C95-A120-D58694B9DB38}"/>
-    <hyperlink ref="F28" r:id="rId9" xr:uid="{EB55229C-F54B-4C46-94E1-24EE1011AE7A}"/>
+    <hyperlink ref="F29" r:id="rId9" xr:uid="{EB55229C-F54B-4C46-94E1-24EE1011AE7A}"/>
     <hyperlink ref="F9" r:id="rId10" xr:uid="{51B52101-2A4A-4111-9EB0-D94FF7DAF0BF}"/>
     <hyperlink ref="F13" r:id="rId11" xr:uid="{5D17CDAE-E94A-464E-BDBE-4D010517E3BC}"/>
     <hyperlink ref="F14" r:id="rId12" xr:uid="{556B9FF1-B5FF-4C94-B027-5745DB6A4DC2}"/>
     <hyperlink ref="F15" r:id="rId13" display="https://www.ebay.com/itm/174968443925?_trkparms=amclksrc%3DITM%26aid%3D777008%26algo%3DPERSONAL.TOPIC%26ao%3D1%26asc%3D20220705100511%26meid%3D2faa5f1c66e54ff3af69f69cbfe6d567%26pid%3D101524%26rk%3D1%26rkt%3D1%26itm%3D174968443925%26pmt%3D1%26noa%3D1%26pg%3D2380057%26algv%3DRecentlyViewedItemsV2&amp;_trksid=p2380057.c101524.m146925&amp;_trkparms=pageci%3Aca4f6cab-ee8f-11ed-9b33-d2bafba4db3b%7Cparentrq%3A019472791880a69e559fc3aafffefea4%7Ciid%3A1" xr:uid="{24EF6E9B-3278-49A3-92E9-C39691B78F2E}"/>
     <hyperlink ref="F16" r:id="rId14" xr:uid="{1078468C-9681-4B8B-B881-6DF6F32C87FA}"/>
-    <hyperlink ref="F20" r:id="rId15" xr:uid="{A4B0540A-680F-4F3A-A223-E547C41E6857}"/>
+    <hyperlink ref="F21" r:id="rId15" xr:uid="{A4B0540A-680F-4F3A-A223-E547C41E6857}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId16"/>

</xml_diff>